<commit_message>
tested on real ui
</commit_message>
<xml_diff>
--- a/TestData/IdData.xlsx
+++ b/TestData/IdData.xlsx
@@ -8,7 +8,7 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="/Users/liganye/PycharmProjects/AlunaTest/TestData/"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{47F0E415-3288-E34B-B396-CAC22B9F2F49}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{D91186C6-6385-6146-9C61-C2269ACC9F10}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
     <workbookView xWindow="4940" yWindow="1300" windowWidth="19200" windowHeight="14160" xr2:uid="{506C5B70-69DE-AB47-8785-A35BF1CCD761}"/>
   </bookViews>
@@ -35,7 +35,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="48" uniqueCount="36">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="45" uniqueCount="34">
   <si>
     <t>id</t>
   </si>
@@ -94,9 +94,6 @@
     <t>Female</t>
   </si>
   <si>
-    <t>INVALID_ID_0</t>
-  </si>
-  <si>
     <t>INVALID_ID_1</t>
   </si>
   <si>
@@ -119,9 +116,6 @@
   </si>
   <si>
     <t>no</t>
-  </si>
-  <si>
-    <t xml:space="preserve"> </t>
   </si>
   <si>
     <t>JUGO1940</t>
@@ -184,10 +178,9 @@
   <cellStyleXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="3">
+  <cellXfs count="2">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
     <xf numFmtId="49" fontId="0" fillId="0" borderId="0" xfId="0" applyNumberFormat="1"/>
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" quotePrefix="1"/>
   </cellXfs>
   <cellStyles count="1">
     <cellStyle name="Normal" xfId="0" builtinId="0"/>
@@ -502,7 +495,7 @@
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{1BFCB89B-7209-1143-9551-E91A19959FBE}">
-  <dimension ref="A1:F12"/>
+  <dimension ref="A1:F11"/>
   <sheetFormatPr baseColWidth="10" defaultRowHeight="16" x14ac:dyDescent="0.2"/>
   <cols>
     <col min="1" max="1" width="12.5" bestFit="1" customWidth="1"/>
@@ -596,11 +589,11 @@
       <c r="A5" t="s">
         <v>19</v>
       </c>
-      <c r="B5" s="2" t="s">
-        <v>28</v>
+      <c r="B5" t="s">
+        <v>27</v>
       </c>
       <c r="C5" t="s">
-        <v>27</v>
+        <v>26</v>
       </c>
     </row>
     <row r="6" spans="1:6" x14ac:dyDescent="0.2">
@@ -608,10 +601,10 @@
         <v>20</v>
       </c>
       <c r="B6" t="s">
-        <v>29</v>
+        <v>28</v>
       </c>
       <c r="C6" t="s">
-        <v>27</v>
+        <v>26</v>
       </c>
     </row>
     <row r="7" spans="1:6" x14ac:dyDescent="0.2">
@@ -619,10 +612,10 @@
         <v>21</v>
       </c>
       <c r="B7" t="s">
-        <v>30</v>
+        <v>29</v>
       </c>
       <c r="C7" t="s">
-        <v>27</v>
+        <v>26</v>
       </c>
     </row>
     <row r="8" spans="1:6" x14ac:dyDescent="0.2">
@@ -630,10 +623,10 @@
         <v>22</v>
       </c>
       <c r="B8" t="s">
-        <v>31</v>
+        <v>30</v>
       </c>
       <c r="C8" t="s">
-        <v>27</v>
+        <v>26</v>
       </c>
     </row>
     <row r="9" spans="1:6" x14ac:dyDescent="0.2">
@@ -641,10 +634,10 @@
         <v>23</v>
       </c>
       <c r="B9" t="s">
-        <v>32</v>
+        <v>31</v>
       </c>
       <c r="C9" t="s">
-        <v>27</v>
+        <v>26</v>
       </c>
     </row>
     <row r="10" spans="1:6" x14ac:dyDescent="0.2">
@@ -652,10 +645,10 @@
         <v>24</v>
       </c>
       <c r="B10" t="s">
-        <v>33</v>
+        <v>32</v>
       </c>
       <c r="C10" t="s">
-        <v>27</v>
+        <v>26</v>
       </c>
     </row>
     <row r="11" spans="1:6" x14ac:dyDescent="0.2">
@@ -663,21 +656,10 @@
         <v>25</v>
       </c>
       <c r="B11" t="s">
-        <v>34</v>
+        <v>33</v>
       </c>
       <c r="C11" t="s">
-        <v>27</v>
-      </c>
-    </row>
-    <row r="12" spans="1:6" x14ac:dyDescent="0.2">
-      <c r="A12" t="s">
         <v>26</v>
-      </c>
-      <c r="B12" t="s">
-        <v>35</v>
-      </c>
-      <c r="C12" t="s">
-        <v>27</v>
       </c>
     </row>
   </sheetData>

</xml_diff>